<commit_message>
graficas de antares y ras algethi
</commit_message>
<xml_diff>
--- a/Datos de fuentes externas/Smith.xlsx
+++ b/Datos de fuentes externas/Smith.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jessi Dani\OneDrive - Universidad de los andes\TESIS\Datos de fuentes externas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jessi Dani\OneDrive - Universidad de los andes\TESIS\Tesis\Datos de fuentes externas\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB2F9DC2-E766-4D42-A4BC-C4CF6E3FE5B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -320,7 +320,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -349,18 +349,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -373,23 +361,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -398,9 +383,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -729,21 +711,21 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="12"/>
-      <c r="F2" s="10" t="s">
+      <c r="C2" s="17"/>
+      <c r="D2" s="18"/>
+      <c r="F2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="11"/>
-      <c r="H2" s="12"/>
-      <c r="J2" s="24" t="s">
+      <c r="G2" s="17"/>
+      <c r="H2" s="18"/>
+      <c r="J2" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="K2" s="25"/>
-      <c r="L2" s="26"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="21"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B3" s="7" t="s">
@@ -755,22 +737,22 @@
       <c r="D3" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="H3" s="17" t="s">
+      <c r="H3" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="15" t="s">
+      <c r="J3" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="K3" s="16" t="s">
+      <c r="K3" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="L3" s="17" t="s">
+      <c r="L3" s="13" t="s">
         <v>2</v>
       </c>
     </row>
@@ -784,22 +766,22 @@
       <c r="D4" s="3">
         <v>-6.01</v>
       </c>
-      <c r="F4" s="18">
+      <c r="F4" s="2">
         <v>6072</v>
       </c>
-      <c r="G4" s="13">
+      <c r="G4" s="1">
         <v>-6.74</v>
       </c>
-      <c r="H4" s="19">
+      <c r="H4" s="3">
         <v>-11.6</v>
       </c>
-      <c r="J4" s="18">
+      <c r="J4" s="2">
         <v>6663</v>
       </c>
-      <c r="K4" s="13">
+      <c r="K4" s="1">
         <v>-32.119999999999997</v>
       </c>
-      <c r="L4" s="19">
+      <c r="L4" s="3">
         <v>-9.49</v>
       </c>
     </row>
@@ -813,22 +795,22 @@
       <c r="D5" s="3">
         <v>-6.77</v>
       </c>
-      <c r="F5" s="18">
+      <c r="F5" s="2">
         <v>6083</v>
       </c>
-      <c r="G5" s="13">
+      <c r="G5" s="1">
         <v>-6.38</v>
       </c>
-      <c r="H5" s="20">
+      <c r="H5" s="14">
         <v>-10.77</v>
       </c>
-      <c r="J5" s="27">
+      <c r="J5" s="15">
         <v>6670</v>
       </c>
-      <c r="K5" s="14">
+      <c r="K5" s="10">
         <v>-33.07</v>
       </c>
-      <c r="L5" s="20">
+      <c r="L5" s="14">
         <v>-6.48</v>
       </c>
     </row>
@@ -842,22 +824,22 @@
       <c r="D6" s="3">
         <v>-5.97</v>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="2">
         <v>6106</v>
       </c>
-      <c r="G6" s="13">
+      <c r="G6" s="1">
         <v>-5.85</v>
       </c>
-      <c r="H6" s="19">
+      <c r="H6" s="3">
         <v>-11.98</v>
       </c>
-      <c r="J6" s="18">
+      <c r="J6" s="2">
         <v>6673</v>
       </c>
-      <c r="K6" s="13">
+      <c r="K6" s="1">
         <v>-33.119999999999997</v>
       </c>
-      <c r="L6" s="19">
+      <c r="L6" s="3">
         <v>-6.43</v>
       </c>
     </row>
@@ -871,22 +853,22 @@
       <c r="D7" s="3">
         <v>-8.39</v>
       </c>
-      <c r="F7" s="18">
+      <c r="F7" s="2">
         <v>6125</v>
       </c>
-      <c r="G7" s="13">
+      <c r="G7" s="1">
         <v>-5.96</v>
       </c>
-      <c r="H7" s="19">
+      <c r="H7" s="3">
         <v>-11.09</v>
       </c>
-      <c r="J7" s="18">
+      <c r="J7" s="2">
         <v>6675</v>
       </c>
-      <c r="K7" s="13">
+      <c r="K7" s="1">
         <v>-33.31</v>
       </c>
-      <c r="L7" s="19">
+      <c r="L7" s="3">
         <v>-5.73</v>
       </c>
     </row>
@@ -900,22 +882,22 @@
       <c r="D8" s="3">
         <v>-10.66</v>
       </c>
-      <c r="F8" s="18">
+      <c r="F8" s="2">
         <v>6159</v>
       </c>
-      <c r="G8" s="13">
+      <c r="G8" s="1">
         <v>-5.12</v>
       </c>
-      <c r="H8" s="19">
+      <c r="H8" s="3">
         <v>-11.18</v>
       </c>
-      <c r="J8" s="18">
+      <c r="J8" s="2">
         <v>6698</v>
       </c>
-      <c r="K8" s="13">
+      <c r="K8" s="1">
         <v>-35.08</v>
       </c>
-      <c r="L8" s="19">
+      <c r="L8" s="3">
         <v>-2.5099999999999998</v>
       </c>
     </row>
@@ -929,22 +911,22 @@
       <c r="D9" s="3">
         <v>-11.99</v>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="2">
         <v>6206</v>
       </c>
-      <c r="G9" s="13">
+      <c r="G9" s="1">
         <v>-5.37</v>
       </c>
-      <c r="H9" s="19">
+      <c r="H9" s="3">
         <v>-10.5</v>
       </c>
-      <c r="J9" s="18">
+      <c r="J9" s="2">
         <v>6699</v>
       </c>
-      <c r="K9" s="13">
+      <c r="K9" s="1">
         <v>-37.840000000000003</v>
       </c>
-      <c r="L9" s="19">
+      <c r="L9" s="3">
         <v>-2.23</v>
       </c>
     </row>
@@ -958,22 +940,22 @@
       <c r="D10" s="3">
         <v>-4.92</v>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="2">
         <v>6213</v>
       </c>
-      <c r="G10" s="13">
+      <c r="G10" s="1">
         <v>-5.73</v>
       </c>
-      <c r="H10" s="19">
+      <c r="H10" s="3">
         <v>-9.61</v>
       </c>
-      <c r="J10" s="18">
+      <c r="J10" s="2">
         <v>6700</v>
       </c>
-      <c r="K10" s="13">
+      <c r="K10" s="1">
         <v>-35.130000000000003</v>
       </c>
-      <c r="L10" s="19">
+      <c r="L10" s="3">
         <v>-2.39</v>
       </c>
     </row>
@@ -987,22 +969,22 @@
       <c r="D11" s="3">
         <v>-3.9</v>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="2">
         <v>6222</v>
       </c>
-      <c r="G11" s="13">
+      <c r="G11" s="1">
         <v>-5.99</v>
       </c>
-      <c r="H11" s="19">
+      <c r="H11" s="3">
         <v>-11.06</v>
       </c>
-      <c r="J11" s="18">
+      <c r="J11" s="2">
         <v>6701</v>
       </c>
-      <c r="K11" s="13">
+      <c r="K11" s="1">
         <v>-36.01</v>
       </c>
-      <c r="L11" s="19">
+      <c r="L11" s="3">
         <v>-1.3</v>
       </c>
     </row>
@@ -1016,22 +998,22 @@
       <c r="D12" s="3">
         <v>-4.13</v>
       </c>
-      <c r="F12" s="18">
+      <c r="F12" s="2">
         <v>6235</v>
       </c>
-      <c r="G12" s="13">
+      <c r="G12" s="1">
         <v>-5.55</v>
       </c>
-      <c r="H12" s="19">
+      <c r="H12" s="3">
         <v>-11.26</v>
       </c>
-      <c r="J12" s="18">
+      <c r="J12" s="2">
         <v>6702</v>
       </c>
-      <c r="K12" s="13">
+      <c r="K12" s="1">
         <v>-35.380000000000003</v>
       </c>
-      <c r="L12" s="19">
+      <c r="L12" s="3">
         <v>-0.86</v>
       </c>
     </row>
@@ -1045,22 +1027,22 @@
       <c r="D13" s="3">
         <v>-5.7</v>
       </c>
-      <c r="F13" s="18">
+      <c r="F13" s="2">
         <v>6249</v>
       </c>
-      <c r="G13" s="13">
+      <c r="G13" s="1">
         <v>-5.61</v>
       </c>
-      <c r="H13" s="19">
+      <c r="H13" s="3">
         <v>-10.32</v>
       </c>
-      <c r="J13" s="18">
+      <c r="J13" s="2">
         <v>6883</v>
       </c>
-      <c r="K13" s="13">
+      <c r="K13" s="1">
         <v>-27.93</v>
       </c>
-      <c r="L13" s="19">
+      <c r="L13" s="3">
         <v>-6.04</v>
       </c>
     </row>
@@ -1074,22 +1056,22 @@
       <c r="D14" s="3">
         <v>-6.43</v>
       </c>
-      <c r="F14" s="18">
+      <c r="F14" s="2">
         <v>6271</v>
       </c>
-      <c r="G14" s="13">
+      <c r="G14" s="1">
         <v>-6.56</v>
       </c>
-      <c r="H14" s="19">
+      <c r="H14" s="3">
         <v>-10.5</v>
       </c>
-      <c r="J14" s="18">
+      <c r="J14" s="2">
         <v>6885</v>
       </c>
-      <c r="K14" s="13">
+      <c r="K14" s="1">
         <v>-29.28</v>
       </c>
-      <c r="L14" s="19">
+      <c r="L14" s="3">
         <v>-4.18</v>
       </c>
     </row>
@@ -1103,22 +1085,22 @@
       <c r="D15" s="3">
         <v>-6.38</v>
       </c>
-      <c r="F15" s="18">
+      <c r="F15" s="2">
         <v>6279</v>
       </c>
-      <c r="G15" s="13">
+      <c r="G15" s="1">
         <v>-6.89</v>
       </c>
-      <c r="H15" s="19">
+      <c r="H15" s="3">
         <v>-15.24</v>
       </c>
-      <c r="J15" s="18">
+      <c r="J15" s="2">
         <v>6912</v>
       </c>
-      <c r="K15" s="13">
+      <c r="K15" s="1">
         <v>-24.62</v>
       </c>
-      <c r="L15" s="19">
+      <c r="L15" s="3">
         <v>-6.55</v>
       </c>
     </row>
@@ -1132,22 +1114,22 @@
       <c r="D16" s="3">
         <v>-4.3099999999999996</v>
       </c>
-      <c r="F16" s="18">
+      <c r="F16" s="2">
         <v>6301</v>
       </c>
-      <c r="G16" s="13">
+      <c r="G16" s="1">
         <v>-9.15</v>
       </c>
-      <c r="H16" s="19">
+      <c r="H16" s="3">
         <v>-10.58</v>
       </c>
-      <c r="J16" s="18">
+      <c r="J16" s="2">
         <v>6913</v>
       </c>
-      <c r="K16" s="13">
+      <c r="K16" s="1">
         <v>-24.96</v>
       </c>
-      <c r="L16" s="19">
+      <c r="L16" s="3">
         <v>-6.31</v>
       </c>
     </row>
@@ -1161,22 +1143,22 @@
       <c r="D17" s="3">
         <v>-5.27</v>
       </c>
-      <c r="F17" s="18">
+      <c r="F17" s="2">
         <v>6322</v>
       </c>
-      <c r="G17" s="13">
+      <c r="G17" s="1">
         <v>-8.86</v>
       </c>
-      <c r="H17" s="19">
+      <c r="H17" s="3">
         <v>-10.78</v>
       </c>
-      <c r="J17" s="18">
+      <c r="J17" s="2">
         <v>6948</v>
       </c>
-      <c r="K17" s="13">
+      <c r="K17" s="1">
         <v>-27.34</v>
       </c>
-      <c r="L17" s="19">
+      <c r="L17" s="3">
         <v>-4.25</v>
       </c>
     </row>
@@ -1190,22 +1172,22 @@
       <c r="D18" s="3">
         <v>-4.4800000000000004</v>
       </c>
-      <c r="F18" s="18">
+      <c r="F18" s="2">
         <v>6330</v>
       </c>
-      <c r="G18" s="13">
+      <c r="G18" s="1">
         <v>-5.75</v>
       </c>
-      <c r="H18" s="19">
+      <c r="H18" s="3">
         <v>-10.59</v>
       </c>
-      <c r="J18" s="18">
+      <c r="J18" s="2">
         <v>6949</v>
       </c>
-      <c r="K18" s="13">
+      <c r="K18" s="1">
         <v>-26.36</v>
       </c>
-      <c r="L18" s="19">
+      <c r="L18" s="3">
         <v>-3.63</v>
       </c>
     </row>
@@ -1219,22 +1201,22 @@
       <c r="D19" s="3">
         <v>-4.91</v>
       </c>
-      <c r="F19" s="18">
+      <c r="F19" s="2">
         <v>6331</v>
       </c>
-      <c r="G19" s="13">
+      <c r="G19" s="1">
         <v>-6.67</v>
       </c>
-      <c r="H19" s="19">
+      <c r="H19" s="3">
         <v>-10.23</v>
       </c>
-      <c r="J19" s="18">
+      <c r="J19" s="2">
         <v>6958</v>
       </c>
-      <c r="K19" s="13">
+      <c r="K19" s="1">
         <v>-27.28</v>
       </c>
-      <c r="L19" s="19">
+      <c r="L19" s="3">
         <v>-3.31</v>
       </c>
     </row>
@@ -1248,22 +1230,22 @@
       <c r="D20" s="3">
         <v>-7.61</v>
       </c>
-      <c r="F20" s="18">
+      <c r="F20" s="2">
         <v>6341</v>
       </c>
-      <c r="G20" s="13">
+      <c r="G20" s="1">
         <v>-7.17</v>
       </c>
-      <c r="H20" s="19">
+      <c r="H20" s="3">
         <v>-11.4</v>
       </c>
-      <c r="J20" s="18">
+      <c r="J20" s="2">
         <v>7012</v>
       </c>
-      <c r="K20" s="13">
+      <c r="K20" s="1">
         <v>-27.71</v>
       </c>
-      <c r="L20" s="19">
+      <c r="L20" s="3">
         <v>-2.16</v>
       </c>
     </row>
@@ -1277,22 +1259,22 @@
       <c r="D21" s="3">
         <v>-5.84</v>
       </c>
-      <c r="F21" s="18">
+      <c r="F21" s="2">
         <v>6474</v>
       </c>
-      <c r="G21" s="13">
+      <c r="G21" s="1">
         <v>-4.5599999999999996</v>
       </c>
-      <c r="H21" s="19">
+      <c r="H21" s="3">
         <v>-14.29</v>
       </c>
-      <c r="J21" s="18">
+      <c r="J21" s="2">
         <v>7199</v>
       </c>
-      <c r="K21" s="13">
+      <c r="K21" s="1">
         <v>-29.58</v>
       </c>
-      <c r="L21" s="19">
+      <c r="L21" s="3">
         <v>-4.1100000000000003</v>
       </c>
     </row>
@@ -1306,22 +1288,22 @@
       <c r="D22" s="3">
         <v>-7.02</v>
       </c>
-      <c r="F22" s="18">
+      <c r="F22" s="2">
         <v>6475</v>
       </c>
-      <c r="G22" s="13">
+      <c r="G22" s="1">
         <v>-5.9</v>
       </c>
-      <c r="H22" s="19">
+      <c r="H22" s="3">
         <v>-11.95</v>
       </c>
-      <c r="J22" s="18">
+      <c r="J22" s="2">
         <v>7207</v>
       </c>
-      <c r="K22" s="13">
+      <c r="K22" s="1">
         <v>-28.71</v>
       </c>
-      <c r="L22" s="19">
+      <c r="L22" s="3">
         <v>-3.16</v>
       </c>
     </row>
@@ -1335,22 +1317,22 @@
       <c r="D23" s="3">
         <v>-6.74</v>
       </c>
-      <c r="F23" s="18">
+      <c r="F23" s="2">
         <v>6478</v>
       </c>
-      <c r="G23" s="13">
+      <c r="G23" s="1">
         <v>-5.14</v>
       </c>
-      <c r="H23" s="19">
+      <c r="H23" s="3">
         <v>-12.74</v>
       </c>
-      <c r="J23" s="18">
+      <c r="J23" s="2">
         <v>7217</v>
       </c>
-      <c r="K23" s="13">
+      <c r="K23" s="1">
         <v>-28</v>
       </c>
-      <c r="L23" s="19">
+      <c r="L23" s="3">
         <v>-4.3099999999999996</v>
       </c>
     </row>
@@ -1364,22 +1346,22 @@
       <c r="D24" s="3">
         <v>-5.99</v>
       </c>
-      <c r="F24" s="18">
+      <c r="F24" s="2">
         <v>6479</v>
       </c>
-      <c r="G24" s="13">
+      <c r="G24" s="1">
         <v>-4.29</v>
       </c>
-      <c r="H24" s="19">
+      <c r="H24" s="3">
         <v>-13.12</v>
       </c>
-      <c r="J24" s="18">
+      <c r="J24" s="2">
         <v>7221</v>
       </c>
-      <c r="K24" s="13">
+      <c r="K24" s="1">
         <v>-29.8</v>
       </c>
-      <c r="L24" s="19">
+      <c r="L24" s="3">
         <v>-0.92</v>
       </c>
     </row>
@@ -1393,22 +1375,22 @@
       <c r="D25" s="3">
         <v>-5.9</v>
       </c>
-      <c r="F25" s="18">
+      <c r="F25" s="2">
         <v>6484</v>
       </c>
-      <c r="G25" s="13">
+      <c r="G25" s="1">
         <v>-4.5999999999999996</v>
       </c>
-      <c r="H25" s="19">
+      <c r="H25" s="3">
         <v>-12.79</v>
       </c>
-      <c r="J25" s="18">
+      <c r="J25" s="2">
         <v>7234</v>
       </c>
-      <c r="K25" s="13">
+      <c r="K25" s="1">
         <v>-32.44</v>
       </c>
-      <c r="L25" s="19">
+      <c r="L25" s="3">
         <v>-1.18</v>
       </c>
     </row>
@@ -1422,22 +1404,22 @@
       <c r="D26" s="3">
         <v>-6.38</v>
       </c>
-      <c r="F26" s="18">
+      <c r="F26" s="2">
         <v>6485</v>
       </c>
-      <c r="G26" s="13">
+      <c r="G26" s="1">
         <v>-4.1100000000000003</v>
       </c>
-      <c r="H26" s="19">
+      <c r="H26" s="3">
         <v>-13.26</v>
       </c>
-      <c r="J26" s="18">
+      <c r="J26" s="2">
         <v>7260</v>
       </c>
-      <c r="K26" s="13">
+      <c r="K26" s="1">
         <v>-27.89</v>
       </c>
-      <c r="L26" s="19">
+      <c r="L26" s="3">
         <v>-1.57</v>
       </c>
     </row>
@@ -1451,22 +1433,22 @@
       <c r="D27" s="3">
         <v>-6.26</v>
       </c>
-      <c r="F27" s="18">
+      <c r="F27" s="2">
         <v>6492</v>
       </c>
-      <c r="G27" s="13">
+      <c r="G27" s="1">
         <v>-5.37</v>
       </c>
-      <c r="H27" s="19">
+      <c r="H27" s="3">
         <v>-13.77</v>
       </c>
-      <c r="J27" s="18">
+      <c r="J27" s="2">
         <v>7289</v>
       </c>
-      <c r="K27" s="13">
+      <c r="K27" s="1">
         <v>-27.76</v>
       </c>
-      <c r="L27" s="19">
+      <c r="L27" s="3">
         <v>-3.82</v>
       </c>
     </row>
@@ -1480,22 +1462,22 @@
       <c r="D28" s="3">
         <v>-3.76</v>
       </c>
-      <c r="F28" s="18">
+      <c r="F28" s="2">
         <v>6493</v>
       </c>
-      <c r="G28" s="13">
+      <c r="G28" s="1">
         <v>-3.18</v>
       </c>
-      <c r="H28" s="19">
+      <c r="H28" s="3">
         <v>-11.91</v>
       </c>
-      <c r="J28" s="18">
+      <c r="J28" s="2">
         <v>7339</v>
       </c>
-      <c r="K28" s="13">
+      <c r="K28" s="1">
         <v>-30.79</v>
       </c>
-      <c r="L28" s="19">
+      <c r="L28" s="3">
         <v>0.42</v>
       </c>
     </row>
@@ -1509,22 +1491,22 @@
       <c r="D29" s="3">
         <v>-5.07</v>
       </c>
-      <c r="F29" s="18">
+      <c r="F29" s="2">
         <v>6494</v>
       </c>
-      <c r="G29" s="13">
+      <c r="G29" s="1">
         <v>-4.41</v>
       </c>
-      <c r="H29" s="19">
+      <c r="H29" s="3">
         <v>-12.62</v>
       </c>
-      <c r="J29" s="18">
+      <c r="J29" s="2">
         <v>7537</v>
       </c>
-      <c r="K29" s="13">
+      <c r="K29" s="1">
         <v>-31.03</v>
       </c>
-      <c r="L29" s="19">
+      <c r="L29" s="3">
         <v>-2.69</v>
       </c>
     </row>
@@ -1538,22 +1520,22 @@
       <c r="D30" s="3">
         <v>-5.95</v>
       </c>
-      <c r="F30" s="18">
+      <c r="F30" s="2">
         <v>6495</v>
       </c>
-      <c r="G30" s="13">
+      <c r="G30" s="1">
         <v>-5.73</v>
       </c>
-      <c r="H30" s="19">
+      <c r="H30" s="3">
         <v>-12.37</v>
       </c>
-      <c r="J30" s="18">
+      <c r="J30" s="2">
         <v>7541</v>
       </c>
-      <c r="K30" s="13">
+      <c r="K30" s="1">
         <v>-31.77</v>
       </c>
-      <c r="L30" s="19">
+      <c r="L30" s="3">
         <v>-0.99</v>
       </c>
     </row>
@@ -1567,22 +1549,22 @@
       <c r="D31" s="3">
         <v>-5.5</v>
       </c>
-      <c r="F31" s="18">
+      <c r="F31" s="2">
         <v>6496</v>
       </c>
-      <c r="G31" s="13">
+      <c r="G31" s="1">
         <v>-4.78</v>
       </c>
-      <c r="H31" s="19">
+      <c r="H31" s="3">
         <v>-12.85</v>
       </c>
-      <c r="J31" s="18">
+      <c r="J31" s="2">
         <v>7568</v>
       </c>
-      <c r="K31" s="13">
+      <c r="K31" s="1">
         <v>-31.86</v>
       </c>
-      <c r="L31" s="19">
+      <c r="L31" s="3">
         <v>-1.21</v>
       </c>
     </row>
@@ -1596,22 +1578,22 @@
       <c r="D32" s="3">
         <v>-5.24</v>
       </c>
-      <c r="F32" s="18">
+      <c r="F32" s="2">
         <v>6497</v>
       </c>
-      <c r="G32" s="13">
+      <c r="G32" s="1">
         <v>-5.18</v>
       </c>
-      <c r="H32" s="19">
+      <c r="H32" s="3">
         <v>-12.89</v>
       </c>
-      <c r="J32" s="18">
+      <c r="J32" s="2">
         <v>7581</v>
       </c>
-      <c r="K32" s="13">
+      <c r="K32" s="1">
         <v>-30.39</v>
       </c>
-      <c r="L32" s="19">
+      <c r="L32" s="3">
         <v>-1.28</v>
       </c>
     </row>
@@ -1625,22 +1607,22 @@
       <c r="D33" s="3">
         <v>-5.24</v>
       </c>
-      <c r="F33" s="18">
+      <c r="F33" s="2">
         <v>6504</v>
       </c>
-      <c r="G33" s="13">
+      <c r="G33" s="1">
         <v>-6.27</v>
       </c>
-      <c r="H33" s="19">
+      <c r="H33" s="3">
         <v>-10.71</v>
       </c>
-      <c r="J33" s="18">
+      <c r="J33" s="2">
         <v>7599</v>
       </c>
-      <c r="K33" s="13">
+      <c r="K33" s="1">
         <v>-29.92</v>
       </c>
-      <c r="L33" s="19">
+      <c r="L33" s="3">
         <v>-2.08</v>
       </c>
     </row>
@@ -1654,22 +1636,22 @@
       <c r="D34" s="3">
         <v>-4.47</v>
       </c>
-      <c r="F34" s="18">
+      <c r="F34" s="2">
         <v>6529</v>
       </c>
-      <c r="G34" s="13">
+      <c r="G34" s="1">
         <v>-6.78</v>
       </c>
-      <c r="H34" s="19">
+      <c r="H34" s="3">
         <v>-10.45</v>
       </c>
-      <c r="J34" s="18">
+      <c r="J34" s="2">
         <v>7604</v>
       </c>
-      <c r="K34" s="13">
+      <c r="K34" s="1">
         <v>-29.11</v>
       </c>
-      <c r="L34" s="19">
+      <c r="L34" s="3">
         <v>-1.99</v>
       </c>
     </row>
@@ -1683,22 +1665,22 @@
       <c r="D35" s="3">
         <v>-4.1900000000000004</v>
       </c>
-      <c r="F35" s="18">
+      <c r="F35" s="2">
         <v>6538</v>
       </c>
-      <c r="G35" s="13">
+      <c r="G35" s="1">
         <v>-4.92</v>
       </c>
-      <c r="H35" s="19">
+      <c r="H35" s="3">
         <v>-12.76</v>
       </c>
-      <c r="J35" s="18">
+      <c r="J35" s="2">
         <v>7608</v>
       </c>
-      <c r="K35" s="13">
+      <c r="K35" s="1">
         <v>-29.44</v>
       </c>
-      <c r="L35" s="19">
+      <c r="L35" s="3">
         <v>-0.31</v>
       </c>
     </row>
@@ -1712,22 +1694,22 @@
       <c r="D36" s="3">
         <v>-4.83</v>
       </c>
-      <c r="F36" s="18">
+      <c r="F36" s="2">
         <v>6539</v>
       </c>
-      <c r="G36" s="13">
+      <c r="G36" s="1">
         <v>-4.43</v>
       </c>
-      <c r="H36" s="19">
+      <c r="H36" s="3">
         <v>-12.01</v>
       </c>
-      <c r="J36" s="18">
+      <c r="J36" s="2">
         <v>7613</v>
       </c>
-      <c r="K36" s="13">
+      <c r="K36" s="1">
         <v>-31.11</v>
       </c>
-      <c r="L36" s="19">
+      <c r="L36" s="3">
         <v>-1.51</v>
       </c>
     </row>
@@ -1741,22 +1723,22 @@
       <c r="D37" s="3">
         <v>-4.6399999999999997</v>
       </c>
-      <c r="F37" s="18">
+      <c r="F37" s="2">
         <v>6547</v>
       </c>
-      <c r="G37" s="13">
+      <c r="G37" s="1">
         <v>-4.67</v>
       </c>
-      <c r="H37" s="19">
+      <c r="H37" s="3">
         <v>-15.54</v>
       </c>
-      <c r="J37" s="21">
+      <c r="J37" s="4">
         <v>7626</v>
       </c>
-      <c r="K37" s="22">
+      <c r="K37" s="5">
         <v>-31.31</v>
       </c>
-      <c r="L37" s="23">
+      <c r="L37" s="6">
         <v>-0.73</v>
       </c>
     </row>
@@ -1770,13 +1752,13 @@
       <c r="D38" s="3">
         <v>-4.8099999999999996</v>
       </c>
-      <c r="F38" s="18">
+      <c r="F38" s="2">
         <v>6555</v>
       </c>
-      <c r="G38" s="13">
+      <c r="G38" s="1">
         <v>-4.03</v>
       </c>
-      <c r="H38" s="19">
+      <c r="H38" s="3">
         <v>-12.21</v>
       </c>
     </row>
@@ -1790,13 +1772,13 @@
       <c r="D39" s="3">
         <v>-5.78</v>
       </c>
-      <c r="F39" s="18">
+      <c r="F39" s="2">
         <v>6564</v>
       </c>
-      <c r="G39" s="13">
+      <c r="G39" s="1">
         <v>-4.26</v>
       </c>
-      <c r="H39" s="19">
+      <c r="H39" s="3">
         <v>-12.9</v>
       </c>
     </row>
@@ -1810,13 +1792,13 @@
       <c r="D40" s="3">
         <v>-3.1</v>
       </c>
-      <c r="F40" s="18">
+      <c r="F40" s="2">
         <v>6585</v>
       </c>
-      <c r="G40" s="13">
+      <c r="G40" s="1">
         <v>-7.66</v>
       </c>
-      <c r="H40" s="19">
+      <c r="H40" s="3">
         <v>-12.87</v>
       </c>
     </row>
@@ -1830,13 +1812,13 @@
       <c r="D41" s="3">
         <v>-3.25</v>
       </c>
-      <c r="F41" s="18">
+      <c r="F41" s="2">
         <v>6663</v>
       </c>
-      <c r="G41" s="13">
+      <c r="G41" s="1">
         <v>-3.42</v>
       </c>
-      <c r="H41" s="19">
+      <c r="H41" s="3">
         <v>-15.51</v>
       </c>
     </row>
@@ -1850,13 +1832,13 @@
       <c r="D42" s="3">
         <v>-2.64</v>
       </c>
-      <c r="F42" s="18">
+      <c r="F42" s="2">
         <v>6670</v>
       </c>
-      <c r="G42" s="13">
+      <c r="G42" s="1">
         <v>-4.74</v>
       </c>
-      <c r="H42" s="19">
+      <c r="H42" s="3">
         <v>-12.81</v>
       </c>
     </row>
@@ -1870,13 +1852,13 @@
       <c r="D43" s="3">
         <v>-1.83</v>
       </c>
-      <c r="F43" s="18">
+      <c r="F43" s="2">
         <v>6673</v>
       </c>
-      <c r="G43" s="13">
+      <c r="G43" s="1">
         <v>-5.09</v>
       </c>
-      <c r="H43" s="19">
+      <c r="H43" s="3">
         <v>-15.03</v>
       </c>
     </row>
@@ -1890,13 +1872,13 @@
       <c r="D44" s="3">
         <v>-2.36</v>
       </c>
-      <c r="F44" s="18">
+      <c r="F44" s="2">
         <v>6675</v>
       </c>
-      <c r="G44" s="13">
+      <c r="G44" s="1">
         <v>-4.55</v>
       </c>
-      <c r="H44" s="19">
+      <c r="H44" s="3">
         <v>-12.72</v>
       </c>
     </row>
@@ -1910,13 +1892,13 @@
       <c r="D45" s="3">
         <v>-3.24</v>
       </c>
-      <c r="F45" s="18">
+      <c r="F45" s="2">
         <v>6698</v>
       </c>
-      <c r="G45" s="13">
+      <c r="G45" s="1">
         <v>-3.38</v>
       </c>
-      <c r="H45" s="19">
+      <c r="H45" s="3">
         <v>-13.53</v>
       </c>
     </row>
@@ -1930,13 +1912,13 @@
       <c r="D46" s="3">
         <v>-3.17</v>
       </c>
-      <c r="F46" s="18">
+      <c r="F46" s="2">
         <v>6699</v>
       </c>
-      <c r="G46" s="13">
+      <c r="G46" s="1">
         <v>-3.81</v>
       </c>
-      <c r="H46" s="19">
+      <c r="H46" s="3">
         <v>-14.56</v>
       </c>
     </row>
@@ -1950,13 +1932,13 @@
       <c r="D47" s="3">
         <v>-3.83</v>
       </c>
-      <c r="F47" s="18">
+      <c r="F47" s="2">
         <v>6700</v>
       </c>
-      <c r="G47" s="13">
+      <c r="G47" s="1">
         <v>-2.96</v>
       </c>
-      <c r="H47" s="19">
+      <c r="H47" s="3">
         <v>-13.33</v>
       </c>
     </row>
@@ -1970,13 +1952,13 @@
       <c r="D48" s="3">
         <v>-3.67</v>
       </c>
-      <c r="F48" s="18">
+      <c r="F48" s="2">
         <v>6701</v>
       </c>
-      <c r="G48" s="13">
+      <c r="G48" s="1">
         <v>-3.86</v>
       </c>
-      <c r="H48" s="19">
+      <c r="H48" s="3">
         <v>-13.02</v>
       </c>
     </row>
@@ -1990,13 +1972,13 @@
       <c r="D49" s="3">
         <v>-2.94</v>
       </c>
-      <c r="F49" s="18">
+      <c r="F49" s="2">
         <v>6702</v>
       </c>
-      <c r="G49" s="13">
+      <c r="G49" s="1">
         <v>-3.33</v>
       </c>
-      <c r="H49" s="19">
+      <c r="H49" s="3">
         <v>-12.4</v>
       </c>
     </row>
@@ -2010,13 +1992,13 @@
       <c r="D50" s="3">
         <v>-5.69</v>
       </c>
-      <c r="F50" s="18">
+      <c r="F50" s="2">
         <v>6820</v>
       </c>
-      <c r="G50" s="13">
+      <c r="G50" s="1">
         <v>-3.18</v>
       </c>
-      <c r="H50" s="19">
+      <c r="H50" s="3">
         <v>-12</v>
       </c>
     </row>
@@ -2030,13 +2012,13 @@
       <c r="D51" s="3">
         <v>-3.06</v>
       </c>
-      <c r="F51" s="18">
+      <c r="F51" s="2">
         <v>6828</v>
       </c>
-      <c r="G51" s="13">
+      <c r="G51" s="1">
         <v>-3.35</v>
       </c>
-      <c r="H51" s="19">
+      <c r="H51" s="3">
         <v>-11.23</v>
       </c>
     </row>
@@ -2050,13 +2032,13 @@
       <c r="D52" s="3">
         <v>-3.97</v>
       </c>
-      <c r="F52" s="18">
+      <c r="F52" s="2">
         <v>6883</v>
       </c>
-      <c r="G52" s="13">
+      <c r="G52" s="1">
         <v>-1.68</v>
       </c>
-      <c r="H52" s="19">
+      <c r="H52" s="3">
         <v>-11.38</v>
       </c>
     </row>
@@ -2070,13 +2052,13 @@
       <c r="D53" s="3">
         <v>-4.83</v>
       </c>
-      <c r="F53" s="18">
+      <c r="F53" s="2">
         <v>6885</v>
       </c>
-      <c r="G53" s="13">
+      <c r="G53" s="1">
         <v>-2.21</v>
       </c>
-      <c r="H53" s="19">
+      <c r="H53" s="3">
         <v>-10.94</v>
       </c>
     </row>
@@ -2090,13 +2072,13 @@
       <c r="D54" s="3">
         <v>-1.47</v>
       </c>
-      <c r="F54" s="18">
+      <c r="F54" s="2">
         <v>6912</v>
       </c>
-      <c r="G54" s="13">
+      <c r="G54" s="1">
         <v>-0.66</v>
       </c>
-      <c r="H54" s="19">
+      <c r="H54" s="3">
         <v>-9.1999999999999993</v>
       </c>
     </row>
@@ -2110,13 +2092,13 @@
       <c r="D55" s="3">
         <v>-4.37</v>
       </c>
-      <c r="F55" s="18">
+      <c r="F55" s="2">
         <v>6913</v>
       </c>
-      <c r="G55" s="13">
+      <c r="G55" s="1">
         <v>-1.1299999999999999</v>
       </c>
-      <c r="H55" s="19">
+      <c r="H55" s="3">
         <v>-9.2200000000000006</v>
       </c>
     </row>
@@ -2130,13 +2112,13 @@
       <c r="D56" s="3">
         <v>-3.59</v>
       </c>
-      <c r="F56" s="18">
+      <c r="F56" s="2">
         <v>6948</v>
       </c>
-      <c r="G56" s="13">
+      <c r="G56" s="1">
         <v>-0.18</v>
       </c>
-      <c r="H56" s="19">
+      <c r="H56" s="3">
         <v>-11.72</v>
       </c>
     </row>
@@ -2150,13 +2132,13 @@
       <c r="D57" s="3">
         <v>0.14000000000000001</v>
       </c>
-      <c r="F57" s="18">
+      <c r="F57" s="2">
         <v>6949</v>
       </c>
-      <c r="G57" s="13">
+      <c r="G57" s="1">
         <v>-0.33</v>
       </c>
-      <c r="H57" s="19">
+      <c r="H57" s="3">
         <v>-9.82</v>
       </c>
     </row>
@@ -2170,13 +2152,13 @@
       <c r="D58" s="3">
         <v>-4.66</v>
       </c>
-      <c r="F58" s="18">
+      <c r="F58" s="2">
         <v>6958</v>
       </c>
-      <c r="G58" s="13">
+      <c r="G58" s="1">
         <v>-0.76</v>
       </c>
-      <c r="H58" s="19">
+      <c r="H58" s="3">
         <v>-11.09</v>
       </c>
     </row>
@@ -2190,13 +2172,13 @@
       <c r="D59" s="3">
         <v>-4.93</v>
       </c>
-      <c r="F59" s="18">
+      <c r="F59" s="2">
         <v>7199</v>
       </c>
-      <c r="G59" s="13">
+      <c r="G59" s="1">
         <v>-3.02</v>
       </c>
-      <c r="H59" s="19">
+      <c r="H59" s="3">
         <v>-8.69</v>
       </c>
     </row>
@@ -2210,13 +2192,13 @@
       <c r="D60" s="3">
         <v>1.59</v>
       </c>
-      <c r="F60" s="18">
+      <c r="F60" s="2">
         <v>7207</v>
       </c>
-      <c r="G60" s="13">
+      <c r="G60" s="1">
         <v>-2.58</v>
       </c>
-      <c r="H60" s="19">
+      <c r="H60" s="3">
         <v>-8.58</v>
       </c>
     </row>
@@ -2230,13 +2212,13 @@
       <c r="D61" s="3">
         <v>-4.58</v>
       </c>
-      <c r="F61" s="18">
+      <c r="F61" s="2">
         <v>7217</v>
       </c>
-      <c r="G61" s="13">
+      <c r="G61" s="1">
         <v>-1.68</v>
       </c>
-      <c r="H61" s="19">
+      <c r="H61" s="3">
         <v>-9.8000000000000007</v>
       </c>
     </row>
@@ -2250,13 +2232,13 @@
       <c r="D62" s="3">
         <v>0.22</v>
       </c>
-      <c r="F62" s="18">
+      <c r="F62" s="2">
         <v>7221</v>
       </c>
-      <c r="G62" s="13">
+      <c r="G62" s="1">
         <v>-0.35</v>
       </c>
-      <c r="H62" s="19">
+      <c r="H62" s="3">
         <v>-8.7899999999999991</v>
       </c>
     </row>
@@ -2270,13 +2252,13 @@
       <c r="D63" s="3">
         <v>0.2</v>
       </c>
-      <c r="F63" s="18">
+      <c r="F63" s="2">
         <v>7234</v>
       </c>
-      <c r="G63" s="13">
+      <c r="G63" s="1">
         <v>1.18</v>
       </c>
-      <c r="H63" s="19">
+      <c r="H63" s="3">
         <v>-13.05</v>
       </c>
     </row>
@@ -2290,13 +2272,13 @@
       <c r="D64" s="3">
         <v>-0.3</v>
       </c>
-      <c r="F64" s="18">
+      <c r="F64" s="2">
         <v>7260</v>
       </c>
-      <c r="G64" s="13">
+      <c r="G64" s="1">
         <v>1.19</v>
       </c>
-      <c r="H64" s="19">
+      <c r="H64" s="3">
         <v>-10.36</v>
       </c>
     </row>
@@ -2310,13 +2292,13 @@
       <c r="D65" s="3">
         <v>-0.91</v>
       </c>
-      <c r="F65" s="18">
+      <c r="F65" s="2">
         <v>7289</v>
       </c>
-      <c r="G65" s="13">
+      <c r="G65" s="1">
         <v>-1.87</v>
       </c>
-      <c r="H65" s="19">
+      <c r="H65" s="3">
         <v>-7.02</v>
       </c>
     </row>
@@ -2330,13 +2312,13 @@
       <c r="D66" s="3">
         <v>-1.44</v>
       </c>
-      <c r="F66" s="18">
+      <c r="F66" s="2">
         <v>7298</v>
       </c>
-      <c r="G66" s="13">
+      <c r="G66" s="1">
         <v>-1.95</v>
       </c>
-      <c r="H66" s="19">
+      <c r="H66" s="3">
         <v>-4.87</v>
       </c>
     </row>
@@ -2350,13 +2332,13 @@
       <c r="D67" s="3">
         <v>0.26</v>
       </c>
-      <c r="F67" s="18">
+      <c r="F67" s="2">
         <v>7339</v>
       </c>
-      <c r="G67" s="13">
+      <c r="G67" s="1">
         <v>-3.3</v>
       </c>
-      <c r="H67" s="19">
+      <c r="H67" s="3">
         <v>-6.94</v>
       </c>
     </row>
@@ -2370,13 +2352,13 @@
       <c r="D68" s="3">
         <v>-0.12</v>
       </c>
-      <c r="F68" s="18">
+      <c r="F68" s="2">
         <v>7537</v>
       </c>
-      <c r="G68" s="13">
+      <c r="G68" s="1">
         <v>-5.64</v>
       </c>
-      <c r="H68" s="19">
+      <c r="H68" s="3">
         <v>-4.5599999999999996</v>
       </c>
     </row>
@@ -2390,13 +2372,13 @@
       <c r="D69" s="3">
         <v>6.22</v>
       </c>
-      <c r="F69" s="18">
+      <c r="F69" s="2">
         <v>7541</v>
       </c>
-      <c r="G69" s="13">
+      <c r="G69" s="1">
         <v>-6</v>
       </c>
-      <c r="H69" s="19">
+      <c r="H69" s="3">
         <v>-4.21</v>
       </c>
     </row>
@@ -2410,13 +2392,13 @@
       <c r="D70" s="3">
         <v>2.64</v>
       </c>
-      <c r="F70" s="18">
+      <c r="F70" s="2">
         <v>7568</v>
       </c>
-      <c r="G70" s="13">
+      <c r="G70" s="1">
         <v>-4.07</v>
       </c>
-      <c r="H70" s="19">
+      <c r="H70" s="3">
         <v>-5.0599999999999996</v>
       </c>
     </row>
@@ -2430,13 +2412,13 @@
       <c r="D71" s="3">
         <v>2.5099999999999998</v>
       </c>
-      <c r="F71" s="18">
+      <c r="F71" s="2">
         <v>7581</v>
       </c>
-      <c r="G71" s="13">
+      <c r="G71" s="1">
         <v>-3.42</v>
       </c>
-      <c r="H71" s="19">
+      <c r="H71" s="3">
         <v>-5.04</v>
       </c>
     </row>
@@ -2450,13 +2432,13 @@
       <c r="D72" s="3">
         <v>-0.78</v>
       </c>
-      <c r="F72" s="18">
+      <c r="F72" s="2">
         <v>7599</v>
       </c>
-      <c r="G72" s="13">
+      <c r="G72" s="1">
         <v>-1.69</v>
       </c>
-      <c r="H72" s="19">
+      <c r="H72" s="3">
         <v>-6.54</v>
       </c>
     </row>
@@ -2470,13 +2452,13 @@
       <c r="D73" s="3">
         <v>-2.5</v>
       </c>
-      <c r="F73" s="18">
+      <c r="F73" s="2">
         <v>7604</v>
       </c>
-      <c r="G73" s="13">
+      <c r="G73" s="1">
         <v>-2.56</v>
       </c>
-      <c r="H73" s="19">
+      <c r="H73" s="3">
         <v>-5.32</v>
       </c>
     </row>
@@ -2490,13 +2472,13 @@
       <c r="D74" s="3">
         <v>-3.16</v>
       </c>
-      <c r="F74" s="18">
+      <c r="F74" s="2">
         <v>7608</v>
       </c>
-      <c r="G74" s="13">
+      <c r="G74" s="1">
         <v>-1.86</v>
       </c>
-      <c r="H74" s="19">
+      <c r="H74" s="3">
         <v>-4.7300000000000004</v>
       </c>
     </row>
@@ -2510,13 +2492,13 @@
       <c r="D75" s="3">
         <v>-2.33</v>
       </c>
-      <c r="F75" s="18">
+      <c r="F75" s="2">
         <v>7613</v>
       </c>
-      <c r="G75" s="13">
+      <c r="G75" s="1">
         <v>-2.4</v>
       </c>
-      <c r="H75" s="19">
+      <c r="H75" s="3">
         <v>-5.72</v>
       </c>
     </row>
@@ -2530,13 +2512,13 @@
       <c r="D76" s="3">
         <v>-2.62</v>
       </c>
-      <c r="F76" s="18">
+      <c r="F76" s="2">
         <v>7626</v>
       </c>
-      <c r="G76" s="13">
+      <c r="G76" s="1">
         <v>-2.99</v>
       </c>
-      <c r="H76" s="19">
+      <c r="H76" s="3">
         <v>-3.34</v>
       </c>
     </row>
@@ -2550,13 +2532,13 @@
       <c r="D77" s="3">
         <v>-3.27</v>
       </c>
-      <c r="F77" s="21">
+      <c r="F77" s="4">
         <v>7631</v>
       </c>
-      <c r="G77" s="22">
+      <c r="G77" s="5">
         <v>-2.31</v>
       </c>
-      <c r="H77" s="23">
+      <c r="H77" s="6">
         <v>-5.82</v>
       </c>
     </row>

</xml_diff>